<commit_message>
Updated pin assignments in spreadsheet
</commit_message>
<xml_diff>
--- a/hardware/docs/stm32l1_pins.xlsx
+++ b/hardware/docs/stm32l1_pins.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="25516"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="80" windowWidth="25600" windowHeight="17540" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="17540" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Pins" sheetId="5" r:id="rId1"/>
@@ -25,7 +25,7 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <connection id="1" name="stm32l1_pins.txt" type="6" refreshedVersion="0" background="1" saveData="1">
-    <textPr fileType="mac" codePage="10000" sourceFile="Macintosh HD:Users:user:projects:alti:hardware:stm32l1_pins.txt" tab="0" space="1" consecutive="1">
+    <textPr fileType="mac" sourceFile="Macintosh HD:Users:user:projects:alti:hardware:stm32l1_pins.txt" tab="0" space="1" consecutive="1">
       <textFields count="11">
         <textField/>
         <textField/>
@@ -42,7 +42,7 @@
     </textPr>
   </connection>
   <connection id="2" name="stm32l1_pins.txt1" type="6" refreshedVersion="0" background="1" saveData="1">
-    <textPr fileType="mac" codePage="10000" sourceFile="Macintosh HD:Users:user:projects:alti:hardware:stm32l1_pins.txt" tab="0" space="1" consecutive="1">
+    <textPr fileType="mac" sourceFile="Macintosh HD:Users:user:projects:alti:hardware:stm32l1_pins.txt" tab="0" space="1" consecutive="1">
       <textFields count="11">
         <textField/>
         <textField/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="418">
   <si>
     <t>Name</t>
   </si>
@@ -865,9 +865,6 @@
     <t>PA11</t>
   </si>
   <si>
-    <t>USART1_CTS/</t>
-  </si>
-  <si>
     <t>B8</t>
   </si>
   <si>
@@ -1175,13 +1172,157 @@
   </si>
   <si>
     <t>PH1-OSC_OUT</t>
+  </si>
+  <si>
+    <t>Alti Assignment</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>SWD</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>+3V</t>
+  </si>
+  <si>
+    <t>SWCLK</t>
+  </si>
+  <si>
+    <t>-SWCLK</t>
+  </si>
+  <si>
+    <t>USART1_CTS</t>
+  </si>
+  <si>
+    <t>USB_DM</t>
+  </si>
+  <si>
+    <t>USB_HEADER</t>
+  </si>
+  <si>
+    <t>SWD_HEADER</t>
+  </si>
+  <si>
+    <t>LSE</t>
+  </si>
+  <si>
+    <t>HSE</t>
+  </si>
+  <si>
+    <t>16MHz xtal</t>
+  </si>
+  <si>
+    <t>32k xtal</t>
+  </si>
+  <si>
+    <t>RESET</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>?????????</t>
+  </si>
+  <si>
+    <t>RDYN</t>
+  </si>
+  <si>
+    <t>REQN</t>
+  </si>
+  <si>
+    <t>nrf8001_RSET</t>
+  </si>
+  <si>
+    <t>Can potentially share this with other IC's</t>
+  </si>
+  <si>
+    <t>SPI2_MISO</t>
+  </si>
+  <si>
+    <t>SPI2_MOSI</t>
+  </si>
+  <si>
+    <t>nrf8001_enable</t>
+  </si>
+  <si>
+    <t>nrf8001_SCK</t>
+  </si>
+  <si>
+    <t>nrf8001_MISO</t>
+  </si>
+  <si>
+    <t>nrf8001_MOSI</t>
+  </si>
+  <si>
+    <t>nrf8001_REQN</t>
+  </si>
+  <si>
+    <t>nrf8001_RDYN</t>
+  </si>
+  <si>
+    <t>MS5611_SCK</t>
+  </si>
+  <si>
+    <t>MS5611_MISO</t>
+  </si>
+  <si>
+    <t>MS5611_MOSI</t>
+  </si>
+  <si>
+    <t>ms5611_enable</t>
+  </si>
+  <si>
+    <t>AT45DB321E_SCK</t>
+  </si>
+  <si>
+    <t>AT45DB321E_MISO</t>
+  </si>
+  <si>
+    <t>AT45DB321E_MOSI</t>
+  </si>
+  <si>
+    <t>BOOT0 (tie to gnd or vcc)</t>
+  </si>
+  <si>
+    <t>WARN LED select</t>
+  </si>
+  <si>
+    <t>WARN LED enable</t>
+  </si>
+  <si>
+    <t>BMX055 SDA</t>
+  </si>
+  <si>
+    <t>BMX055 SCLK</t>
+  </si>
+  <si>
+    <t>BMX055 EN</t>
+  </si>
+  <si>
+    <t>STATUS LED</t>
+  </si>
+  <si>
+    <t>Piezzo Out</t>
+  </si>
+  <si>
+    <t>Piezzo Enable</t>
+  </si>
+  <si>
+    <t>NRF8001_Enable</t>
+  </si>
+  <si>
+    <t>AT45DB321E_enable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1197,13 +1338,59 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1215,14 +1402,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="9">
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1557,23 +1769,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1" enableFormatConditionsCalculation="0"/>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:O112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1640625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" customWidth="1"/>
     <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="49.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="45.1640625" customWidth="1"/>
     <col min="11" max="11" width="33.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.5" customWidth="1"/>
+    <col min="13" max="13" width="28.5" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1607,8 +1822,14 @@
       <c r="K1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="M1" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>6</v>
       </c>
@@ -1621,26 +1842,32 @@
       <c r="D2" t="s">
         <v>37</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="3">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="M2" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>7</v>
       </c>
@@ -1653,29 +1880,32 @@
       <c r="D3" t="s">
         <v>41</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="3">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
-        <v>366</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="J3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>8</v>
       </c>
@@ -1688,29 +1918,36 @@
       <c r="D4" t="s">
         <v>43</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="3">
         <v>3</v>
       </c>
-      <c r="F4" t="s">
-        <v>367</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="F4" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="J4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="J4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="M4" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="O4" s="7"/>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>9</v>
       </c>
@@ -1723,29 +1960,36 @@
       <c r="D5" t="s">
         <v>45</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="3">
         <v>4</v>
       </c>
-      <c r="F5" t="s">
-        <v>368</v>
-      </c>
-      <c r="G5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="F5" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J5" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="J5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="M5" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="O5" s="7"/>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>12</v>
       </c>
@@ -1758,29 +2002,36 @@
       <c r="D6" t="s">
         <v>50</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="3">
         <v>5</v>
       </c>
-      <c r="F6" t="s">
-        <v>369</v>
-      </c>
-      <c r="G6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="F6" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="J6" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="J6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="M6" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="O6" s="7"/>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>13</v>
       </c>
@@ -1793,29 +2044,36 @@
       <c r="D7" t="s">
         <v>53</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="3">
         <v>6</v>
       </c>
-      <c r="F7" t="s">
-        <v>370</v>
-      </c>
-      <c r="G7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="F7" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="J7" t="s">
-        <v>17</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="J7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="M7" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="O7" s="7"/>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>14</v>
       </c>
@@ -1828,29 +2086,36 @@
       <c r="D8" t="s">
         <v>56</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="3">
         <v>7</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="G8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="J8" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="J8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="O8" s="7"/>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>19</v>
       </c>
@@ -1863,29 +2128,34 @@
       <c r="D9" t="s">
         <v>76</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="3">
         <v>8</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="H9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J9" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="J9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>22</v>
       </c>
@@ -1898,29 +2168,34 @@
       <c r="D10" t="s">
         <v>82</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="3">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="H10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="J10" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="J10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>23</v>
       </c>
@@ -1933,29 +2208,32 @@
       <c r="D11" t="s">
         <v>84</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="3">
         <v>10</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="G11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:11">
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>24</v>
       </c>
@@ -1968,29 +2246,32 @@
       <c r="D12" t="s">
         <v>89</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="3">
         <v>11</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G12" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="G12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="13" spans="1:11">
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>25</v>
       </c>
@@ -2003,29 +2284,32 @@
       <c r="D13" t="s">
         <v>94</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="3">
         <v>12</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" t="s">
+      <c r="G13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="14" spans="1:11">
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>26</v>
       </c>
@@ -2038,29 +2322,32 @@
       <c r="D14" t="s">
         <v>99</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="4">
         <v>13</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="G14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="4" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="15" spans="1:11">
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>29</v>
       </c>
@@ -2073,29 +2360,32 @@
       <c r="D15" t="s">
         <v>106</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="4">
         <v>14</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="G15" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="G15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="4" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>30</v>
       </c>
@@ -2108,29 +2398,38 @@
       <c r="D16" t="s">
         <v>111</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="4">
         <v>15</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="G16" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="G16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="4" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="M16" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="N16" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="O16" s="10" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17">
         <v>31</v>
       </c>
@@ -2143,29 +2442,38 @@
       <c r="D17" t="s">
         <v>116</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="4">
         <v>16</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="G17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" t="s">
+      <c r="G17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="K17" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="K17" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="N17" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="O17" s="10" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18">
         <v>32</v>
       </c>
@@ -2178,29 +2486,38 @@
       <c r="D18" t="s">
         <v>120</v>
       </c>
-      <c r="E18">
-        <v>17</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="E18" s="4">
+        <v>17</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G18" t="s">
-        <v>20</v>
-      </c>
-      <c r="H18" t="s">
-        <v>21</v>
-      </c>
-      <c r="I18" t="s">
+      <c r="G18" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="M18" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="O18" s="10" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19">
         <v>35</v>
       </c>
@@ -2213,29 +2530,36 @@
       <c r="D19" t="s">
         <v>135</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="4">
         <v>18</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="G19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="G19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="M19" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="O19" s="7"/>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20">
         <v>36</v>
       </c>
@@ -2248,29 +2572,36 @@
       <c r="D20" t="s">
         <v>140</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="4">
         <v>19</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G20" t="s">
-        <v>20</v>
-      </c>
-      <c r="H20" t="s">
-        <v>21</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="G20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="4" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="M20" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="O20" s="7"/>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21">
         <v>37</v>
       </c>
@@ -2283,29 +2614,38 @@
       <c r="D21" t="s">
         <v>145</v>
       </c>
-      <c r="E21">
-        <v>20</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="E21" s="4">
+        <v>20</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="G21" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="G21" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I21" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="K21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+      <c r="K21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22">
         <v>47</v>
       </c>
@@ -2318,29 +2658,36 @@
       <c r="D22" t="s">
         <v>179</v>
       </c>
-      <c r="E22">
-        <v>21</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="E22" s="4">
+        <v>21</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="G22" t="s">
-        <v>20</v>
-      </c>
-      <c r="H22" t="s">
-        <v>21</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="G22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="K22" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
+      <c r="K22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="O22" s="7"/>
+    </row>
+    <row r="23" spans="1:15">
       <c r="A23">
         <v>48</v>
       </c>
@@ -2353,29 +2700,35 @@
       <c r="D23" t="s">
         <v>183</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="4">
         <v>22</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="G23" t="s">
-        <v>20</v>
-      </c>
-      <c r="H23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="G23" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I23" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="K23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
+      <c r="K23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="N23" s="10" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15">
       <c r="A24">
         <v>49</v>
       </c>
@@ -2388,29 +2741,34 @@
       <c r="D24" t="s">
         <v>187</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="4">
         <v>23</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H24" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="H24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="J24" t="s">
-        <v>17</v>
-      </c>
-      <c r="K24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
+      <c r="J24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
+    </row>
+    <row r="25" spans="1:15">
       <c r="A25">
         <v>50</v>
       </c>
@@ -2423,29 +2781,34 @@
       <c r="D25" t="s">
         <v>190</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="4">
         <v>24</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H25" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="H25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="J25" t="s">
-        <v>17</v>
-      </c>
-      <c r="K25" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+      <c r="J25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+    </row>
+    <row r="26" spans="1:15">
       <c r="A26">
         <v>51</v>
       </c>
@@ -2458,29 +2821,36 @@
       <c r="D26" t="s">
         <v>193</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="5">
         <v>25</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="G26" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" t="s">
-        <v>21</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="G26" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I26" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26" s="5" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="27" spans="1:11">
+      <c r="M26" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="N26" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="O26" s="7"/>
+    </row>
+    <row r="27" spans="1:15">
       <c r="A27">
         <v>52</v>
       </c>
@@ -2493,29 +2863,36 @@
       <c r="D27" t="s">
         <v>198</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="5">
         <v>26</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="G27" t="s">
-        <v>20</v>
-      </c>
-      <c r="H27" t="s">
-        <v>21</v>
-      </c>
-      <c r="I27" t="s">
+      <c r="G27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K27" s="5" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="28" spans="1:11">
+      <c r="M27" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="N27" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="O27" s="7"/>
+    </row>
+    <row r="28" spans="1:15">
       <c r="A28">
         <v>53</v>
       </c>
@@ -2528,29 +2905,36 @@
       <c r="D28" t="s">
         <v>203</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="5">
         <v>27</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="G28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H28" t="s">
-        <v>21</v>
-      </c>
-      <c r="I28" t="s">
+      <c r="G28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I28" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="K28" t="s">
+      <c r="K28" s="5" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="29" spans="1:11">
+      <c r="M28" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="N28" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="O28" s="7"/>
+    </row>
+    <row r="29" spans="1:15">
       <c r="A29">
         <v>54</v>
       </c>
@@ -2563,29 +2947,36 @@
       <c r="D29" t="s">
         <v>208</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="5">
         <v>28</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="G29" t="s">
-        <v>20</v>
-      </c>
-      <c r="H29" t="s">
-        <v>21</v>
-      </c>
-      <c r="I29" t="s">
+      <c r="G29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I29" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29" s="5" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="30" spans="1:11">
+      <c r="M29" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="N29" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="O29" s="7"/>
+    </row>
+    <row r="30" spans="1:15">
       <c r="A30">
         <v>67</v>
       </c>
@@ -2598,29 +2989,32 @@
       <c r="D30" t="s">
         <v>253</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="5">
         <v>29</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="G30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H30" t="s">
-        <v>21</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="G30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I30" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="K30" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+      <c r="K30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+    </row>
+    <row r="31" spans="1:15">
       <c r="A31">
         <v>68</v>
       </c>
@@ -2633,29 +3027,32 @@
       <c r="D31" t="s">
         <v>257</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="5">
         <v>30</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="G31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H31" t="s">
-        <v>21</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="G31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="K31" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+      <c r="K31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31" s="7"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="7"/>
+    </row>
+    <row r="32" spans="1:15">
       <c r="A32">
         <v>69</v>
       </c>
@@ -2668,29 +3065,32 @@
       <c r="D32" t="s">
         <v>261</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="5">
         <v>31</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="G32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H32" t="s">
-        <v>21</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="G32" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I32" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="J32" t="s">
+      <c r="J32" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="K32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
+      <c r="K32" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
+      <c r="O32" s="7"/>
+    </row>
+    <row r="33" spans="1:15">
       <c r="A33">
         <v>70</v>
       </c>
@@ -2703,26 +3103,36 @@
       <c r="D33" t="s">
         <v>265</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="5">
         <v>32</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="G33" t="s">
-        <v>20</v>
-      </c>
-      <c r="H33" t="s">
-        <v>21</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="G33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I33" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="J33" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
+      <c r="J33" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="N33" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="O33" s="7"/>
+    </row>
+    <row r="34" spans="1:15">
       <c r="A34">
         <v>71</v>
       </c>
@@ -2730,34 +3140,41 @@
         <v>45</v>
       </c>
       <c r="C34" t="s">
+        <v>267</v>
+      </c>
+      <c r="D34" t="s">
         <v>268</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" s="5">
+        <v>33</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="E34">
-        <v>33</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="J34" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="G34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H34" t="s">
-        <v>21</v>
-      </c>
-      <c r="I34" t="s">
-        <v>270</v>
-      </c>
-      <c r="J34" t="s">
+      <c r="K34" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="K34" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
+      <c r="M34" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="N34" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="O34" s="7"/>
+    </row>
+    <row r="35" spans="1:15">
       <c r="A35">
         <v>72</v>
       </c>
@@ -2765,34 +3182,41 @@
         <v>46</v>
       </c>
       <c r="C35" t="s">
+        <v>272</v>
+      </c>
+      <c r="D35" t="s">
         <v>273</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" s="5">
+        <v>34</v>
+      </c>
+      <c r="F35" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="E35">
-        <v>34</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I35" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="G35" t="s">
-        <v>20</v>
-      </c>
-      <c r="H35" t="s">
-        <v>21</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="J35" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="J35" t="s">
-        <v>277</v>
-      </c>
-      <c r="K35" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11">
+      <c r="K35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="N35" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="O35" s="7"/>
+    </row>
+    <row r="36" spans="1:15">
       <c r="A36">
         <v>74</v>
       </c>
@@ -2800,34 +3224,39 @@
         <v>47</v>
       </c>
       <c r="C36" t="s">
+        <v>279</v>
+      </c>
+      <c r="D36" t="s">
         <v>280</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" s="5">
+        <v>35</v>
+      </c>
+      <c r="F36" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="E36">
-        <v>35</v>
-      </c>
-      <c r="F36" t="s">
-        <v>282</v>
-      </c>
-      <c r="G36" t="s">
+      <c r="G36" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H36" t="s">
-        <v>17</v>
-      </c>
-      <c r="I36" t="s">
-        <v>282</v>
-      </c>
-      <c r="J36" t="s">
-        <v>17</v>
-      </c>
-      <c r="K36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11">
+      <c r="H36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M36" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
+    </row>
+    <row r="37" spans="1:15">
       <c r="A37">
         <v>75</v>
       </c>
@@ -2835,34 +3264,39 @@
         <v>48</v>
       </c>
       <c r="C37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D37" t="s">
         <v>283</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" s="5">
+        <v>36</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="E37">
-        <v>36</v>
-      </c>
-      <c r="F37" t="s">
-        <v>285</v>
-      </c>
-      <c r="G37" t="s">
+      <c r="G37" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H37" t="s">
-        <v>17</v>
-      </c>
-      <c r="I37" t="s">
-        <v>285</v>
-      </c>
-      <c r="J37" t="s">
-        <v>17</v>
-      </c>
-      <c r="K37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
+      <c r="H37" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
+    </row>
+    <row r="38" spans="1:15">
       <c r="A38">
         <v>76</v>
       </c>
@@ -2870,35 +3304,41 @@
         <v>49</v>
       </c>
       <c r="C38" t="s">
+        <v>285</v>
+      </c>
+      <c r="D38" t="s">
         <v>286</v>
-      </c>
-      <c r="D38" t="s">
-        <v>287</v>
       </c>
       <c r="E38">
         <v>37</v>
       </c>
       <c r="F38" t="s">
+        <v>287</v>
+      </c>
+      <c r="G38" t="s">
+        <v>20</v>
+      </c>
+      <c r="H38" t="s">
+        <v>21</v>
+      </c>
+      <c r="I38" t="s">
         <v>288</v>
       </c>
-      <c r="G38" t="s">
-        <v>20</v>
-      </c>
-      <c r="H38" t="s">
-        <v>21</v>
-      </c>
-      <c r="I38" t="s">
+      <c r="J38" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="K38" t="s">
         <v>289</v>
       </c>
-      <c r="J38" t="e">
-        <f>-SWCLK</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="K38" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11">
+      <c r="M38" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="N38" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="O38" s="7"/>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39">
         <v>77</v>
       </c>
@@ -2906,34 +3346,39 @@
         <v>50</v>
       </c>
       <c r="C39" t="s">
+        <v>290</v>
+      </c>
+      <c r="D39" t="s">
         <v>291</v>
-      </c>
-      <c r="D39" t="s">
-        <v>292</v>
       </c>
       <c r="E39">
         <v>38</v>
       </c>
       <c r="F39" t="s">
+        <v>292</v>
+      </c>
+      <c r="G39" t="s">
+        <v>20</v>
+      </c>
+      <c r="H39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I39" t="s">
         <v>293</v>
       </c>
-      <c r="G39" t="s">
-        <v>20</v>
-      </c>
-      <c r="H39" t="s">
-        <v>21</v>
-      </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>294</v>
       </c>
-      <c r="J39" t="s">
-        <v>295</v>
-      </c>
       <c r="K39" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="40" spans="1:11">
+      <c r="M39" s="7" t="s">
+        <v>415</v>
+      </c>
+      <c r="N39" s="7"/>
+      <c r="O39" s="7"/>
+    </row>
+    <row r="40" spans="1:15">
       <c r="A40">
         <v>89</v>
       </c>
@@ -2941,34 +3386,39 @@
         <v>55</v>
       </c>
       <c r="C40" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D40" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E40">
         <v>39</v>
       </c>
       <c r="F40" t="s">
+        <v>324</v>
+      </c>
+      <c r="G40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H40" t="s">
+        <v>21</v>
+      </c>
+      <c r="I40" t="s">
         <v>325</v>
       </c>
-      <c r="G40" t="s">
-        <v>20</v>
-      </c>
-      <c r="H40" t="s">
-        <v>21</v>
-      </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>326</v>
       </c>
-      <c r="J40" t="s">
+      <c r="K40" t="s">
         <v>327</v>
       </c>
-      <c r="K40" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11">
+      <c r="M40" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="N40" s="7"/>
+      <c r="O40" s="7"/>
+    </row>
+    <row r="41" spans="1:15">
       <c r="A41">
         <v>90</v>
       </c>
@@ -2976,34 +3426,38 @@
         <v>56</v>
       </c>
       <c r="C41" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D41" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E41">
         <v>40</v>
       </c>
       <c r="F41" t="s">
+        <v>329</v>
+      </c>
+      <c r="G41" t="s">
+        <v>20</v>
+      </c>
+      <c r="H41" t="s">
+        <v>21</v>
+      </c>
+      <c r="I41" t="s">
         <v>330</v>
       </c>
-      <c r="G41" t="s">
-        <v>20</v>
-      </c>
-      <c r="H41" t="s">
-        <v>21</v>
-      </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>331</v>
       </c>
-      <c r="J41" t="s">
+      <c r="K41" t="s">
         <v>332</v>
       </c>
-      <c r="K41" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11">
+      <c r="M41" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="N41" s="7"/>
+    </row>
+    <row r="42" spans="1:15">
       <c r="A42">
         <v>91</v>
       </c>
@@ -3011,34 +3465,38 @@
         <v>57</v>
       </c>
       <c r="C42" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D42" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E42">
         <v>41</v>
       </c>
       <c r="F42" t="s">
+        <v>334</v>
+      </c>
+      <c r="G42" t="s">
+        <v>20</v>
+      </c>
+      <c r="H42" t="s">
+        <v>21</v>
+      </c>
+      <c r="I42" t="s">
+        <v>334</v>
+      </c>
+      <c r="J42" t="s">
         <v>335</v>
       </c>
-      <c r="G42" t="s">
-        <v>20</v>
-      </c>
-      <c r="H42" t="s">
-        <v>21</v>
-      </c>
-      <c r="I42" t="s">
-        <v>335</v>
-      </c>
-      <c r="J42" t="s">
-        <v>336</v>
-      </c>
       <c r="K42" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11">
+        <v>332</v>
+      </c>
+      <c r="M42" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="N42" s="7"/>
+    </row>
+    <row r="43" spans="1:15">
       <c r="A43">
         <v>92</v>
       </c>
@@ -3046,31 +3504,35 @@
         <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D43" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E43">
         <v>42</v>
       </c>
       <c r="F43" t="s">
+        <v>337</v>
+      </c>
+      <c r="G43" t="s">
+        <v>20</v>
+      </c>
+      <c r="H43" t="s">
+        <v>21</v>
+      </c>
+      <c r="I43" t="s">
+        <v>337</v>
+      </c>
+      <c r="J43" t="s">
         <v>338</v>
       </c>
-      <c r="G43" t="s">
-        <v>20</v>
-      </c>
-      <c r="H43" t="s">
-        <v>21</v>
-      </c>
-      <c r="I43" t="s">
-        <v>338</v>
-      </c>
-      <c r="J43" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11">
+      <c r="M43" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="N43" s="7"/>
+    </row>
+    <row r="44" spans="1:15">
       <c r="A44">
         <v>93</v>
       </c>
@@ -3078,34 +3540,38 @@
         <v>59</v>
       </c>
       <c r="C44" t="s">
+        <v>339</v>
+      </c>
+      <c r="D44" t="s">
         <v>340</v>
-      </c>
-      <c r="D44" t="s">
-        <v>341</v>
       </c>
       <c r="E44">
         <v>43</v>
       </c>
       <c r="F44" t="s">
+        <v>341</v>
+      </c>
+      <c r="G44" t="s">
+        <v>20</v>
+      </c>
+      <c r="H44" t="s">
+        <v>21</v>
+      </c>
+      <c r="I44" t="s">
+        <v>341</v>
+      </c>
+      <c r="J44" t="s">
         <v>342</v>
       </c>
-      <c r="G44" t="s">
-        <v>20</v>
-      </c>
-      <c r="H44" t="s">
-        <v>21</v>
-      </c>
-      <c r="I44" t="s">
-        <v>342</v>
-      </c>
-      <c r="J44" t="s">
+      <c r="K44" t="s">
         <v>343</v>
       </c>
-      <c r="K44" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11">
+      <c r="M44" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="N44" s="7"/>
+    </row>
+    <row r="45" spans="1:15">
       <c r="A45">
         <v>94</v>
       </c>
@@ -3113,25 +3579,25 @@
         <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D45" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E45">
         <v>44</v>
       </c>
       <c r="F45" t="s">
+        <v>344</v>
+      </c>
+      <c r="G45" t="s">
         <v>345</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>346</v>
       </c>
-      <c r="H45" t="s">
-        <v>347</v>
-      </c>
       <c r="I45" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="J45" t="s">
         <v>17</v>
@@ -3139,8 +3605,12 @@
       <c r="K45" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="46" spans="1:11">
+      <c r="M45" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="N45" s="7"/>
+    </row>
+    <row r="46" spans="1:15">
       <c r="A46">
         <v>95</v>
       </c>
@@ -3148,34 +3618,38 @@
         <v>61</v>
       </c>
       <c r="C46" t="s">
+        <v>347</v>
+      </c>
+      <c r="D46" t="s">
         <v>348</v>
-      </c>
-      <c r="D46" t="s">
-        <v>349</v>
       </c>
       <c r="E46">
         <v>45</v>
       </c>
       <c r="F46" t="s">
+        <v>349</v>
+      </c>
+      <c r="G46" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" t="s">
+        <v>21</v>
+      </c>
+      <c r="I46" t="s">
+        <v>349</v>
+      </c>
+      <c r="J46" t="s">
         <v>350</v>
       </c>
-      <c r="G46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H46" t="s">
-        <v>21</v>
-      </c>
-      <c r="I46" t="s">
-        <v>350</v>
-      </c>
-      <c r="J46" t="s">
-        <v>351</v>
-      </c>
       <c r="K46" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="47" spans="1:11">
+      <c r="M46" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="N46" s="7"/>
+    </row>
+    <row r="47" spans="1:15">
       <c r="A47">
         <v>96</v>
       </c>
@@ -3183,34 +3657,38 @@
         <v>62</v>
       </c>
       <c r="C47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D47" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E47">
         <v>46</v>
       </c>
       <c r="F47" t="s">
+        <v>351</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>21</v>
+      </c>
+      <c r="I47" t="s">
+        <v>351</v>
+      </c>
+      <c r="J47" t="s">
         <v>352</v>
       </c>
-      <c r="G47" t="s">
-        <v>20</v>
-      </c>
-      <c r="H47" t="s">
-        <v>21</v>
-      </c>
-      <c r="I47" t="s">
-        <v>352</v>
-      </c>
-      <c r="J47" t="s">
-        <v>353</v>
-      </c>
       <c r="K47" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="48" spans="1:11">
+      <c r="M47" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="N47" s="7"/>
+    </row>
+    <row r="48" spans="1:15">
       <c r="A48">
         <v>99</v>
       </c>
@@ -3218,16 +3696,16 @@
         <v>63</v>
       </c>
       <c r="C48" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D48" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E48">
         <v>47</v>
       </c>
       <c r="F48" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G48" t="s">
         <v>2</v>
@@ -3236,7 +3714,7 @@
         <v>17</v>
       </c>
       <c r="I48" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J48" t="s">
         <v>17</v>
@@ -3244,8 +3722,12 @@
       <c r="K48" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="49" spans="1:11">
+      <c r="M48" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="N48" s="7"/>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49">
         <v>100</v>
       </c>
@@ -3253,16 +3735,16 @@
         <v>64</v>
       </c>
       <c r="C49" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D49" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E49">
         <v>48</v>
       </c>
       <c r="F49" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G49" t="s">
         <v>2</v>
@@ -3271,7 +3753,7 @@
         <v>17</v>
       </c>
       <c r="I49" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J49" t="s">
         <v>17</v>
@@ -3279,8 +3761,12 @@
       <c r="K49" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" hidden="1">
+      <c r="M49" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="N49" s="7"/>
+    </row>
+    <row r="50" spans="1:14" hidden="1">
       <c r="A50">
         <v>1</v>
       </c>
@@ -3315,7 +3801,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1">
+    <row r="51" spans="1:14" hidden="1">
       <c r="A51">
         <v>2</v>
       </c>
@@ -3350,7 +3836,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1">
+    <row r="52" spans="1:14" hidden="1">
       <c r="A52">
         <v>3</v>
       </c>
@@ -3385,7 +3871,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1">
+    <row r="53" spans="1:14" hidden="1">
       <c r="A53">
         <v>4</v>
       </c>
@@ -3420,7 +3906,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1">
+    <row r="54" spans="1:14" hidden="1">
       <c r="A54">
         <v>5</v>
       </c>
@@ -3455,7 +3941,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:11" hidden="1">
+    <row r="55" spans="1:14" hidden="1">
       <c r="A55">
         <v>10</v>
       </c>
@@ -3490,7 +3976,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:11" hidden="1">
+    <row r="56" spans="1:14" hidden="1">
       <c r="A56">
         <v>11</v>
       </c>
@@ -3525,7 +4011,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1">
+    <row r="57" spans="1:14" hidden="1">
       <c r="A57">
         <v>15</v>
       </c>
@@ -3560,7 +4046,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1">
+    <row r="58" spans="1:14" hidden="1">
       <c r="A58">
         <v>16</v>
       </c>
@@ -3595,7 +4081,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1">
+    <row r="59" spans="1:14" hidden="1">
       <c r="A59">
         <v>17</v>
       </c>
@@ -3630,7 +4116,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1">
+    <row r="60" spans="1:14" hidden="1">
       <c r="A60">
         <v>18</v>
       </c>
@@ -3666,7 +4152,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1">
+    <row r="61" spans="1:14" hidden="1">
       <c r="A61">
         <v>20</v>
       </c>
@@ -3701,7 +4187,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1">
+    <row r="62" spans="1:14" hidden="1">
       <c r="A62">
         <v>21</v>
       </c>
@@ -3736,7 +4222,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1">
+    <row r="63" spans="1:14" hidden="1">
       <c r="A63">
         <v>27</v>
       </c>
@@ -3771,7 +4257,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="64" spans="1:11" hidden="1">
+    <row r="64" spans="1:14" hidden="1">
       <c r="A64">
         <v>28</v>
       </c>
@@ -4625,14 +5111,14 @@
         <v>17</v>
       </c>
       <c r="D88" t="s">
+        <v>277</v>
+      </c>
+      <c r="E88" t="s">
+        <v>17</v>
+      </c>
+      <c r="F88" t="s">
         <v>278</v>
       </c>
-      <c r="E88" t="s">
-        <v>17</v>
-      </c>
-      <c r="F88" t="s">
-        <v>279</v>
-      </c>
       <c r="G88" t="s">
         <v>20</v>
       </c>
@@ -4640,7 +5126,7 @@
         <v>21</v>
       </c>
       <c r="I88" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J88" t="s">
         <v>17</v>
@@ -4657,17 +5143,17 @@
         <v>51</v>
       </c>
       <c r="C89" t="s">
+        <v>295</v>
+      </c>
+      <c r="D89" t="s">
         <v>296</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
+        <v>17</v>
+      </c>
+      <c r="F89" t="s">
         <v>297</v>
       </c>
-      <c r="E89" t="s">
-        <v>17</v>
-      </c>
-      <c r="F89" t="s">
-        <v>298</v>
-      </c>
       <c r="G89" t="s">
         <v>20</v>
       </c>
@@ -4675,10 +5161,10 @@
         <v>21</v>
       </c>
       <c r="I89" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J89" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="K89" t="s">
         <v>17</v>
@@ -4692,17 +5178,17 @@
         <v>52</v>
       </c>
       <c r="C90" t="s">
+        <v>298</v>
+      </c>
+      <c r="D90" t="s">
         <v>299</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
+        <v>17</v>
+      </c>
+      <c r="F90" t="s">
         <v>300</v>
       </c>
-      <c r="E90" t="s">
-        <v>17</v>
-      </c>
-      <c r="F90" t="s">
-        <v>301</v>
-      </c>
       <c r="G90" t="s">
         <v>20</v>
       </c>
@@ -4710,10 +5196,10 @@
         <v>21</v>
       </c>
       <c r="I90" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J90" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="K90" t="s">
         <v>17</v>
@@ -4727,17 +5213,17 @@
         <v>53</v>
       </c>
       <c r="C91" t="s">
+        <v>301</v>
+      </c>
+      <c r="D91" t="s">
         <v>302</v>
       </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
+        <v>17</v>
+      </c>
+      <c r="F91" t="s">
         <v>303</v>
       </c>
-      <c r="E91" t="s">
-        <v>17</v>
-      </c>
-      <c r="F91" t="s">
-        <v>304</v>
-      </c>
       <c r="G91" t="s">
         <v>20</v>
       </c>
@@ -4745,10 +5231,10 @@
         <v>21</v>
       </c>
       <c r="I91" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J91" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K91" t="s">
         <v>17</v>
@@ -4765,25 +5251,25 @@
         <v>17</v>
       </c>
       <c r="D92" t="s">
+        <v>304</v>
+      </c>
+      <c r="E92" t="s">
+        <v>17</v>
+      </c>
+      <c r="F92" t="s">
         <v>305</v>
       </c>
-      <c r="E92" t="s">
-        <v>17</v>
-      </c>
-      <c r="F92" t="s">
+      <c r="G92" t="s">
+        <v>20</v>
+      </c>
+      <c r="H92" t="s">
+        <v>21</v>
+      </c>
+      <c r="I92" t="s">
+        <v>305</v>
+      </c>
+      <c r="J92" t="s">
         <v>306</v>
-      </c>
-      <c r="G92" t="s">
-        <v>20</v>
-      </c>
-      <c r="H92" t="s">
-        <v>21</v>
-      </c>
-      <c r="I92" t="s">
-        <v>306</v>
-      </c>
-      <c r="J92" t="s">
-        <v>307</v>
       </c>
       <c r="K92" t="s">
         <v>17</v>
@@ -4800,25 +5286,25 @@
         <v>17</v>
       </c>
       <c r="D93" t="s">
+        <v>307</v>
+      </c>
+      <c r="E93" t="s">
+        <v>17</v>
+      </c>
+      <c r="F93" t="s">
         <v>308</v>
       </c>
-      <c r="E93" t="s">
-        <v>17</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="G93" t="s">
+        <v>20</v>
+      </c>
+      <c r="H93" t="s">
+        <v>21</v>
+      </c>
+      <c r="I93" t="s">
+        <v>308</v>
+      </c>
+      <c r="J93" t="s">
         <v>309</v>
-      </c>
-      <c r="G93" t="s">
-        <v>20</v>
-      </c>
-      <c r="H93" t="s">
-        <v>21</v>
-      </c>
-      <c r="I93" t="s">
-        <v>309</v>
-      </c>
-      <c r="J93" t="s">
-        <v>310</v>
       </c>
       <c r="K93" t="s">
         <v>17</v>
@@ -4832,7 +5318,7 @@
         <v>54</v>
       </c>
       <c r="C94" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D94" t="s">
         <v>264</v>
@@ -4841,19 +5327,19 @@
         <v>17</v>
       </c>
       <c r="F94" t="s">
+        <v>311</v>
+      </c>
+      <c r="G94" t="s">
+        <v>20</v>
+      </c>
+      <c r="H94" t="s">
+        <v>21</v>
+      </c>
+      <c r="I94" t="s">
+        <v>311</v>
+      </c>
+      <c r="J94" t="s">
         <v>312</v>
-      </c>
-      <c r="G94" t="s">
-        <v>20</v>
-      </c>
-      <c r="H94" t="s">
-        <v>21</v>
-      </c>
-      <c r="I94" t="s">
-        <v>312</v>
-      </c>
-      <c r="J94" t="s">
-        <v>313</v>
       </c>
       <c r="K94" t="s">
         <v>17</v>
@@ -4870,25 +5356,25 @@
         <v>17</v>
       </c>
       <c r="D95" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E95" t="s">
         <v>17</v>
       </c>
       <c r="F95" t="s">
+        <v>313</v>
+      </c>
+      <c r="G95" t="s">
+        <v>20</v>
+      </c>
+      <c r="H95" t="s">
+        <v>21</v>
+      </c>
+      <c r="I95" t="s">
+        <v>313</v>
+      </c>
+      <c r="J95" t="s">
         <v>314</v>
-      </c>
-      <c r="G95" t="s">
-        <v>20</v>
-      </c>
-      <c r="H95" t="s">
-        <v>21</v>
-      </c>
-      <c r="I95" t="s">
-        <v>314</v>
-      </c>
-      <c r="J95" t="s">
-        <v>315</v>
       </c>
       <c r="K95" t="s">
         <v>17</v>
@@ -4905,31 +5391,31 @@
         <v>17</v>
       </c>
       <c r="D96" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E96" t="s">
         <v>17</v>
       </c>
       <c r="F96" t="s">
+        <v>315</v>
+      </c>
+      <c r="G96" t="s">
+        <v>20</v>
+      </c>
+      <c r="H96" t="s">
+        <v>21</v>
+      </c>
+      <c r="I96" t="s">
+        <v>315</v>
+      </c>
+      <c r="J96" t="s">
         <v>316</v>
       </c>
-      <c r="G96" t="s">
-        <v>20</v>
-      </c>
-      <c r="H96" t="s">
-        <v>21</v>
-      </c>
-      <c r="I96" t="s">
-        <v>316</v>
-      </c>
-      <c r="J96" t="s">
-        <v>317</v>
-      </c>
       <c r="K96" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="97" spans="1:11" hidden="1">
+    <row r="97" spans="1:14" hidden="1">
       <c r="A97">
         <v>86</v>
       </c>
@@ -4940,31 +5426,31 @@
         <v>17</v>
       </c>
       <c r="D97" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E97" t="s">
         <v>17</v>
       </c>
       <c r="F97" t="s">
+        <v>317</v>
+      </c>
+      <c r="G97" t="s">
+        <v>20</v>
+      </c>
+      <c r="H97" t="s">
+        <v>21</v>
+      </c>
+      <c r="I97" t="s">
+        <v>317</v>
+      </c>
+      <c r="J97" t="s">
         <v>318</v>
       </c>
-      <c r="G97" t="s">
-        <v>20</v>
-      </c>
-      <c r="H97" t="s">
-        <v>21</v>
-      </c>
-      <c r="I97" t="s">
-        <v>318</v>
-      </c>
-      <c r="J97" t="s">
-        <v>319</v>
-      </c>
       <c r="K97" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="98" spans="1:11" hidden="1">
+    <row r="98" spans="1:14" hidden="1">
       <c r="A98">
         <v>87</v>
       </c>
@@ -4975,31 +5461,31 @@
         <v>17</v>
       </c>
       <c r="D98" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E98" t="s">
         <v>17</v>
       </c>
       <c r="F98" t="s">
+        <v>319</v>
+      </c>
+      <c r="G98" t="s">
+        <v>20</v>
+      </c>
+      <c r="H98" t="s">
+        <v>21</v>
+      </c>
+      <c r="I98" t="s">
+        <v>319</v>
+      </c>
+      <c r="J98" t="s">
         <v>320</v>
       </c>
-      <c r="G98" t="s">
-        <v>20</v>
-      </c>
-      <c r="H98" t="s">
-        <v>21</v>
-      </c>
-      <c r="I98" t="s">
-        <v>320</v>
-      </c>
-      <c r="J98" t="s">
-        <v>321</v>
-      </c>
       <c r="K98" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="99" spans="1:11" hidden="1">
+    <row r="99" spans="1:14" hidden="1">
       <c r="A99">
         <v>88</v>
       </c>
@@ -5010,31 +5496,31 @@
         <v>17</v>
       </c>
       <c r="D99" t="s">
+        <v>321</v>
+      </c>
+      <c r="E99" t="s">
+        <v>17</v>
+      </c>
+      <c r="F99" t="s">
         <v>322</v>
       </c>
-      <c r="E99" t="s">
-        <v>17</v>
-      </c>
-      <c r="F99" t="s">
+      <c r="G99" t="s">
+        <v>20</v>
+      </c>
+      <c r="H99" t="s">
+        <v>21</v>
+      </c>
+      <c r="I99" t="s">
+        <v>322</v>
+      </c>
+      <c r="J99" t="s">
         <v>323</v>
       </c>
-      <c r="G99" t="s">
-        <v>20</v>
-      </c>
-      <c r="H99" t="s">
-        <v>21</v>
-      </c>
-      <c r="I99" t="s">
-        <v>323</v>
-      </c>
-      <c r="J99" t="s">
-        <v>324</v>
-      </c>
       <c r="K99" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="100" spans="1:11" hidden="1">
+    <row r="100" spans="1:14" hidden="1">
       <c r="A100">
         <v>97</v>
       </c>
@@ -5045,31 +5531,31 @@
         <v>17</v>
       </c>
       <c r="D100" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E100" t="s">
         <v>17</v>
       </c>
       <c r="F100" t="s">
+        <v>353</v>
+      </c>
+      <c r="G100" t="s">
+        <v>20</v>
+      </c>
+      <c r="H100" t="s">
+        <v>21</v>
+      </c>
+      <c r="I100" t="s">
+        <v>353</v>
+      </c>
+      <c r="J100" t="s">
         <v>354</v>
       </c>
-      <c r="G100" t="s">
-        <v>20</v>
-      </c>
-      <c r="H100" t="s">
-        <v>21</v>
-      </c>
-      <c r="I100" t="s">
-        <v>354</v>
-      </c>
-      <c r="J100" t="s">
-        <v>355</v>
-      </c>
       <c r="K100" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="101" spans="1:11" hidden="1">
+    <row r="101" spans="1:14" hidden="1">
       <c r="A101">
         <v>98</v>
       </c>
@@ -5086,29 +5572,73 @@
         <v>17</v>
       </c>
       <c r="F101" t="s">
+        <v>355</v>
+      </c>
+      <c r="G101" t="s">
+        <v>20</v>
+      </c>
+      <c r="H101" t="s">
+        <v>21</v>
+      </c>
+      <c r="I101" t="s">
+        <v>355</v>
+      </c>
+      <c r="J101" t="s">
         <v>356</v>
       </c>
-      <c r="G101" t="s">
-        <v>20</v>
-      </c>
-      <c r="H101" t="s">
-        <v>21</v>
-      </c>
-      <c r="I101" t="s">
-        <v>356</v>
-      </c>
-      <c r="J101" t="s">
-        <v>357</v>
-      </c>
       <c r="K101" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="102" spans="1:14">
+      <c r="M102" s="7"/>
+      <c r="N102" s="7"/>
+    </row>
+    <row r="103" spans="1:14">
+      <c r="M103" s="7"/>
+      <c r="N103" s="7"/>
+    </row>
+    <row r="104" spans="1:14">
+      <c r="M104" s="7"/>
+      <c r="N104" s="7"/>
+    </row>
+    <row r="105" spans="1:14">
+      <c r="M105" s="7"/>
+      <c r="N105" s="7"/>
+    </row>
+    <row r="106" spans="1:14">
+      <c r="M106" s="7"/>
+      <c r="N106" s="7"/>
+    </row>
+    <row r="107" spans="1:14">
+      <c r="M107" s="7"/>
+      <c r="N107" s="7"/>
+    </row>
+    <row r="108" spans="1:14">
+      <c r="M108" s="7"/>
+      <c r="N108" s="7"/>
+    </row>
+    <row r="109" spans="1:14">
+      <c r="M109" s="7"/>
+      <c r="N109" s="7"/>
+    </row>
+    <row r="110" spans="1:14">
+      <c r="M110" s="7"/>
+      <c r="N110" s="7"/>
+    </row>
+    <row r="111" spans="1:14">
+      <c r="M111" s="7"/>
+      <c r="N111" s="7"/>
+    </row>
+    <row r="112" spans="1:14">
+      <c r="M112" s="7"/>
+      <c r="N112" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K101">
     <filterColumn colId="4">
       <customFilters>
-        <customFilter operator="notEqual" val="-"/>
+        <customFilter operator="notEqual" val="0"/>
       </customFilters>
     </filterColumn>
     <sortState ref="A2:K101">
@@ -5116,6 +5646,7 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>

</xml_diff>

<commit_message>
Added mcu, connected nrf8001 and flash, new footprint, other changes
</commit_message>
<xml_diff>
--- a/hardware/docs/stm32l1_pins.xlsx
+++ b/hardware/docs/stm32l1_pins.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="25516"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="17540" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25560" windowHeight="28340" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Pins" sheetId="5" r:id="rId1"/>
+    <sheet name="BOM" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Pins!$A$1:$K$101</definedName>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="423">
   <si>
     <t>Name</t>
   </si>
@@ -1204,9 +1205,6 @@
     <t>USB_HEADER</t>
   </si>
   <si>
-    <t>SWD_HEADER</t>
-  </si>
-  <si>
     <t>LSE</t>
   </si>
   <si>
@@ -1228,12 +1226,6 @@
     <t>?????????</t>
   </si>
   <si>
-    <t>RDYN</t>
-  </si>
-  <si>
-    <t>REQN</t>
-  </si>
-  <si>
     <t>nrf8001_RSET</t>
   </si>
   <si>
@@ -1294,28 +1286,52 @@
     <t>WARN LED enable</t>
   </si>
   <si>
-    <t>BMX055 SDA</t>
-  </si>
-  <si>
-    <t>BMX055 SCLK</t>
-  </si>
-  <si>
-    <t>BMX055 EN</t>
-  </si>
-  <si>
     <t>STATUS LED</t>
   </si>
   <si>
-    <t>Piezzo Out</t>
-  </si>
-  <si>
-    <t>Piezzo Enable</t>
-  </si>
-  <si>
     <t>NRF8001_Enable</t>
   </si>
   <si>
     <t>AT45DB321E_enable</t>
+  </si>
+  <si>
+    <t>Mfgr Part #</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>CDC</t>
+  </si>
+  <si>
+    <t>Piezo Out</t>
+  </si>
+  <si>
+    <t>Piezo Enable</t>
+  </si>
+  <si>
+    <t>BMX055 M EN</t>
+  </si>
+  <si>
+    <t>BMX055 A EN</t>
+  </si>
+  <si>
+    <t>BMX055 G EN</t>
+  </si>
+  <si>
+    <t>BMX055 SCK</t>
+  </si>
+  <si>
+    <t>BMX055 MISO</t>
+  </si>
+  <si>
+    <t>BMX055 MOSI</t>
+  </si>
+  <si>
+    <t>BMX055 A Interrupt</t>
   </si>
 </sst>
 </file>
@@ -1355,7 +1371,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1392,6 +1408,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1402,7 +1430,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="9">
+  <cellStyleXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1412,8 +1440,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1425,16 +1467,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="9">
+  <cellStyles count="23">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1786,6 +1844,7 @@
     <col min="12" max="12" width="5.5" customWidth="1"/>
     <col min="13" max="13" width="28.5" customWidth="1"/>
     <col min="14" max="14" width="17.6640625" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1862,7 +1921,7 @@
       </c>
       <c r="K2" s="3"/>
       <c r="M2" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -1940,10 +1999,10 @@
         <v>5</v>
       </c>
       <c r="M4" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="N4" s="7" t="s">
         <v>382</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>383</v>
       </c>
       <c r="O4" s="7"/>
     </row>
@@ -1982,10 +2041,10 @@
         <v>6</v>
       </c>
       <c r="M5" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="N5" s="7" t="s">
         <v>382</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>383</v>
       </c>
       <c r="O5" s="7"/>
     </row>
@@ -2024,10 +2083,10 @@
         <v>52</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O6" s="7"/>
     </row>
@@ -2066,10 +2125,10 @@
         <v>54</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O7" s="7"/>
     </row>
@@ -2108,12 +2167,14 @@
         <v>17</v>
       </c>
       <c r="M8" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="N8" s="7" t="s">
         <v>385</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>386</v>
-      </c>
-      <c r="O8" s="7"/>
+      <c r="O8" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
@@ -2229,7 +2290,9 @@
       <c r="K11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="M11" s="7"/>
+      <c r="M11" s="3" t="s">
+        <v>415</v>
+      </c>
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
     </row>
@@ -2267,7 +2330,9 @@
       <c r="K12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="M12" s="7"/>
+      <c r="M12" s="3" t="s">
+        <v>414</v>
+      </c>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
     </row>
@@ -2306,7 +2371,6 @@
         <v>97</v>
       </c>
       <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15">
@@ -2344,7 +2408,9 @@
         <v>102</v>
       </c>
       <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
+      <c r="N14" s="9" t="s">
+        <v>396</v>
+      </c>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15">
@@ -2382,7 +2448,9 @@
         <v>109</v>
       </c>
       <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
+      <c r="N15" s="9" t="s">
+        <v>395</v>
+      </c>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15">
@@ -2423,10 +2491,10 @@
         <v>171</v>
       </c>
       <c r="N16" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>400</v>
+        <v>392</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -2467,10 +2535,10 @@
         <v>174</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>401</v>
+        <v>393</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -2511,10 +2579,10 @@
         <v>177</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>397</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>402</v>
+        <v>394</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -2551,12 +2619,7 @@
       <c r="K19" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="M19" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="N19" s="9" t="s">
-        <v>399</v>
-      </c>
+      <c r="M19" s="7"/>
       <c r="O19" s="7"/>
     </row>
     <row r="20" spans="1:15">
@@ -2593,12 +2656,7 @@
       <c r="K20" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="M20" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="N20" s="9" t="s">
-        <v>398</v>
-      </c>
+      <c r="M20" s="7"/>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15">
@@ -2639,10 +2697,10 @@
         <v>58</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -2680,10 +2738,10 @@
         <v>17</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="O22" s="7"/>
     </row>
@@ -2722,10 +2780,10 @@
         <v>17</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -2842,13 +2900,9 @@
       <c r="K26" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="M26" s="7" t="s">
-        <v>417</v>
-      </c>
-      <c r="N26" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="O26" s="7"/>
+      <c r="O26" s="12" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27">
@@ -2887,10 +2941,12 @@
       <c r="M27" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="N27" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="O27" s="7"/>
+      <c r="N27" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="O27" s="10" t="s">
+        <v>397</v>
+      </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28">
@@ -2927,12 +2983,14 @@
         <v>206</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="N28" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="O28" s="7"/>
+        <v>389</v>
+      </c>
+      <c r="N28" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="O28" s="10" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29">
@@ -2969,12 +3027,14 @@
         <v>211</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>393</v>
-      </c>
-      <c r="N29" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="O29" s="7"/>
+        <v>390</v>
+      </c>
+      <c r="N29" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="O29" s="10" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30">
@@ -3011,7 +3071,9 @@
         <v>17</v>
       </c>
       <c r="M30" s="7"/>
-      <c r="N30" s="7"/>
+      <c r="N30" s="11" t="s">
+        <v>416</v>
+      </c>
       <c r="O30" s="7"/>
     </row>
     <row r="31" spans="1:15">
@@ -3049,7 +3111,9 @@
         <v>17</v>
       </c>
       <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
+      <c r="N31" s="11" t="s">
+        <v>417</v>
+      </c>
       <c r="O31" s="7"/>
     </row>
     <row r="32" spans="1:15">
@@ -3087,7 +3151,9 @@
         <v>17</v>
       </c>
       <c r="M32" s="7"/>
-      <c r="N32" s="7"/>
+      <c r="N32" s="11" t="s">
+        <v>418</v>
+      </c>
       <c r="O32" s="7"/>
     </row>
     <row r="33" spans="1:15">
@@ -3211,10 +3277,10 @@
       <c r="M35" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="N35" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="O35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36">
@@ -3333,10 +3399,10 @@
       <c r="M38" s="7" t="s">
         <v>375</v>
       </c>
-      <c r="N38" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="O38" s="7"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39">
@@ -3372,11 +3438,11 @@
       <c r="K39" t="s">
         <v>17</v>
       </c>
-      <c r="M39" s="7" t="s">
-        <v>415</v>
-      </c>
+      <c r="M39" s="7"/>
       <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
+      <c r="O39" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40">
@@ -3412,11 +3478,11 @@
       <c r="K40" t="s">
         <v>327</v>
       </c>
-      <c r="M40" s="7" t="s">
-        <v>414</v>
-      </c>
+      <c r="M40" s="7"/>
       <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
+      <c r="O40" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41">
@@ -3453,7 +3519,7 @@
         <v>332</v>
       </c>
       <c r="M41" s="7" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="N41" s="7"/>
     </row>
@@ -3491,9 +3557,7 @@
       <c r="K42" t="s">
         <v>332</v>
       </c>
-      <c r="M42" s="7" t="s">
-        <v>412</v>
-      </c>
+      <c r="M42" s="7"/>
       <c r="N42" s="7"/>
     </row>
     <row r="43" spans="1:15">
@@ -3527,9 +3591,7 @@
       <c r="J43" t="s">
         <v>338</v>
       </c>
-      <c r="M43" s="7" t="s">
-        <v>411</v>
-      </c>
+      <c r="M43" s="7"/>
       <c r="N43" s="7"/>
     </row>
     <row r="44" spans="1:15">
@@ -3566,9 +3628,7 @@
       <c r="K44" t="s">
         <v>343</v>
       </c>
-      <c r="M44" s="7" t="s">
-        <v>410</v>
-      </c>
+      <c r="M44" s="7"/>
       <c r="N44" s="7"/>
     </row>
     <row r="45" spans="1:15">
@@ -3606,7 +3666,7 @@
         <v>17</v>
       </c>
       <c r="M45" s="7" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N45" s="7"/>
     </row>
@@ -3645,7 +3705,7 @@
         <v>17</v>
       </c>
       <c r="M46" s="7" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="N46" s="7"/>
     </row>
@@ -3684,7 +3744,7 @@
         <v>17</v>
       </c>
       <c r="M47" s="7" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="N47" s="7"/>
     </row>
@@ -5632,7 +5692,9 @@
     </row>
     <row r="112" spans="1:14">
       <c r="M112" s="7"/>
-      <c r="N112" s="7"/>
+      <c r="N112" s="11" t="s">
+        <v>422</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K101">
@@ -5653,4 +5715,33 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Lots of hw changes (warn circuits, footprint, etc)
</commit_message>
<xml_diff>
--- a/hardware/docs/stm32l1_pins.xlsx
+++ b/hardware/docs/stm32l1_pins.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="25516"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25640" windowHeight="17540" tabRatio="500"/>
+    <workbookView xWindow="-20" yWindow="0" windowWidth="25640" windowHeight="17540" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Pins" sheetId="5" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="423">
   <si>
     <t>Name</t>
   </si>
@@ -1338,7 +1338,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1366,6 +1366,13 @@
       <u/>
       <sz val="12"/>
       <color theme="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1430,7 +1437,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="35">
+  <cellStyleXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1466,8 +1473,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1481,8 +1492,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="35">
+  <cellStyles count="39">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -1500,6 +1512,8 @@
     <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -1517,6 +1531,8 @@
     <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2800,9 +2816,6 @@
       <c r="M23" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="N23" s="10" t="s">
-        <v>399</v>
-      </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24">
@@ -2917,6 +2930,12 @@
       </c>
       <c r="K26" s="5" t="s">
         <v>196</v>
+      </c>
+      <c r="M26" s="13" t="s">
+        <v>399</v>
+      </c>
+      <c r="N26" s="10" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="27" spans="1:15">

</xml_diff>